<commit_message>
docs: redoing comments in preparation for cargo doc to replace all the markdown files.
</commit_message>
<xml_diff>
--- a/docs/mpmahj features and status.xlsx
+++ b/docs/mpmahj features and status.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\mpmahj\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DD7C0100-5B85-4287-AC33-635F3F274A03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1407FD1C-6A75-406F-A519-DCD9627DC44F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A337DA29-1EF5-4CAB-9594-762ECA37EC0A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="82">
   <si>
     <t>Feature</t>
   </si>
@@ -123,6 +123,165 @@
   </si>
   <si>
     <t>Feature: Dead Hand / Pattern Viability</t>
+  </si>
+  <si>
+    <t>Logic</t>
+  </si>
+  <si>
+    <t>Tile Tracking &amp; Viability Calculation</t>
+  </si>
+  <si>
+    <t>Pattern Difficulty Classification</t>
+  </si>
+  <si>
+    <t>Enhanced Logging &amp; Comparative Analysis</t>
+  </si>
+  <si>
+    <t>Game Activity Log</t>
+  </si>
+  <si>
+    <t>AI Comparison Log</t>
+  </si>
+  <si>
+    <t>Replay System Integration</t>
+  </si>
+  <si>
+    <t>Statistical Tracking</t>
+  </si>
+  <si>
+    <t>Core Rules &amp; Deterministic State</t>
+  </si>
+  <si>
+    <t>Ruleset Configuration</t>
+  </si>
+  <si>
+    <t>Call Priority</t>
+  </si>
+  <si>
+    <t>Joker Rules</t>
+  </si>
+  <si>
+    <t>Scoring &amp; Settlement</t>
+  </si>
+  <si>
+    <t>Deterministic State</t>
+  </si>
+  <si>
+    <t>Multiplayer Stalling Controls</t>
+  </si>
+  <si>
+    <t>Baseline Rules Parity</t>
+  </si>
+  <si>
+    <t>Ruleset Configuration &amp; Metadata</t>
+  </si>
+  <si>
+    <t>Call Priority &amp; Illegal-Move Enforcement</t>
+  </si>
+  <si>
+    <t>Joker Rules &amp; Replacement Draws</t>
+  </si>
+  <si>
+    <t>Scoring, Settlement, and Dealer Rotation</t>
+  </si>
+  <si>
+    <t>Deterministic State Capture</t>
+  </si>
+  <si>
+    <t>Completion Split: Backend Coverage vs Frontend Impact</t>
+  </si>
+  <si>
+    <t>Frontend Impact (what clients must implement)</t>
+  </si>
+  <si>
+    <t>Smart Undo: Where it belongs and what remains</t>
+  </si>
+  <si>
+    <t>Decision-point tagging</t>
+  </si>
+  <si>
+    <t>SmartUndo command/event (small API addition)</t>
+  </si>
+  <si>
+    <t>Bounded history &amp; truncation policy</t>
+  </si>
+  <si>
+    <t>Tests &amp; concurrency checks</t>
+  </si>
+  <si>
+    <t>Optional</t>
+  </si>
+  <si>
+    <t>Additional Features to Consider</t>
+  </si>
+  <si>
+    <t>Defensive Play Analysis</t>
+  </si>
+  <si>
+    <t>Practice Mode Auto-Play</t>
+  </si>
+  <si>
+    <t>Pattern Recommendation Filters</t>
+  </si>
+  <si>
+    <t>Courtesy Pass Negotiation</t>
+  </si>
+  <si>
+    <t>Timer Behavior</t>
+  </si>
+  <si>
+    <t>Feature List</t>
+  </si>
+  <si>
+    <t>State machine design</t>
+  </si>
+  <si>
+    <t>Data models: Tile</t>
+  </si>
+  <si>
+    <t>Data models: Deck / Wall</t>
+  </si>
+  <si>
+    <t>Data models: Hand</t>
+  </si>
+  <si>
+    <t>Data models: Meld</t>
+  </si>
+  <si>
+    <t>Data models: Player</t>
+  </si>
+  <si>
+    <t>Data models: Table (Game State)</t>
+  </si>
+  <si>
+    <t>Data models: Error Types</t>
+  </si>
+  <si>
+    <t>Command / Event System</t>
+  </si>
+  <si>
+    <t>Commands (Player → Server → Core)</t>
+  </si>
+  <si>
+    <t>Events (Server → Client)</t>
+  </si>
+  <si>
+    <t>Command Validation and Results</t>
+  </si>
+  <si>
+    <t>Command Processing Pattern</t>
+  </si>
+  <si>
+    <t>TypeScript Type Generation</t>
+  </si>
+  <si>
+    <t>Event Visibility (Public vs Private)</t>
+  </si>
+  <si>
+    <t>Command Priority and Conflict Resolution</t>
+  </si>
+  <si>
+    <t>The Card Schema</t>
   </si>
 </sst>
 </file>
@@ -173,7 +332,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
@@ -189,6 +348,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -525,14 +687,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA496E7E-C5F5-44C6-A21D-5971EBD7BE23}">
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:F68"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="53.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="9.140625" style="2"/>
+    <col min="6" max="6" width="40" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -542,122 +705,176 @@
       <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="F1" s="4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="F2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="F3" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="F4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="F5" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="F6" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="F7" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="F8" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="F9" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="F10" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="F11" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="F12" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="F13" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="F14" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="F15" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>18</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="F16" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="F17" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="F18" s="7" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>20</v>
       </c>
@@ -665,7 +882,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>5</v>
       </c>
@@ -673,7 +890,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>21</v>
       </c>
@@ -681,7 +898,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>22</v>
       </c>
@@ -689,47 +906,238 @@
         <v>8</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
         <v>28</v>
       </c>
     </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" s="6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A48" s="6" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A52" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A53" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A54" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A55" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A57" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A58" s="6" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A59" s="6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A60" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A61" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A62" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A63" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A64" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A65" s="6" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A66" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A67" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A68" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>